<commit_message>
Fix FATF baseline provenance after failed refresh
Require a successful manifest status before treating a retained snapshot as current data in the workbook and FATF verifier. Fail closed on unavailable or invalid status and validation errors.

Put the baseline warning first, wrap the note, add provenance regression coverage, and correct the existing 2026-10-24 attachment without changing its list data.
</commit_message>
<xml_diff>
--- a/public/downloads/公开名单-CPI-离岸-FATF_20261024.xlsx
+++ b/public/downloads/公开名单-CPI-离岸-FATF_20261024.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -120,6 +120,9 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5059,10 +5062,10 @@
     <col width="44" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>来源: FATF — High-Risk Jurisdictions subject to a Call for Action(黑) / Jurisdictions under Increased Monitoring(灰) · 与本次官方抓取一致（同一期 2026-06），采用法务确认口径，名单日期 2026-06-19（法务维护的基线） · 抓取尝试: 2026-10-24</t>
+    <row r="1" ht="54" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>⚠ 本次抓取失败，使用法务基线（非本次抓取） · 名单日期: 2026-06-19（法务维护的基线） · 抓取尝试: 2026-10-24 · 来源: FATF — High-Risk Jurisdictions subject to a Call for Action(黑) / Jurisdictions under Increased Monitoring(灰)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>

</xml_diff>